<commit_message>
minor change in scenario data
</commit_message>
<xml_diff>
--- a/data/scenarios/food_as_industry.xlsx
+++ b/data/scenarios/food_as_industry.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="11550" activeTab="5"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="18360" windowHeight="6615" firstSheet="1" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Regions" sheetId="7" r:id="rId1"/>
@@ -5989,7 +5989,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.7109375" bestFit="1" customWidth="1"/>
@@ -5998,7 +5998,7 @@
     <col min="4" max="10" width="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>105</v>
       </c>
@@ -6030,7 +6030,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>102</v>
       </c>
@@ -6057,7 +6057,7 @@
         <v>0.83058399999999988</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>104</v>
       </c>
@@ -6082,12 +6082,6 @@
       <c r="J3" s="3">
         <f>H3*(1-0.06)</f>
         <v>0.83058399999999988</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="M7">
-        <f>1-0.83</f>
-        <v>0.17000000000000004</v>
       </c>
     </row>
   </sheetData>

</xml_diff>